<commit_message>
Update runsetup.xlsx fixture for basswood 2026-07-01
</commit_message>
<xml_diff>
--- a/tests/fixtures/basswood_2026-07-01/runsetup.xlsx
+++ b/tests/fixtures/basswood_2026-07-01/runsetup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://baillielumber-my.sharepoint.com/personal/bhanke_baillie_com/Documents/Projects/comact-runsetup-translator/tests/fixtures/basswood_2026-07-01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B2BE603-0DD6-4D35-AFFE-90462E4D228A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CAE152B-5E05-4975-B24B-E09EBF3D2311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2310" yWindow="2310" windowWidth="19190" windowHeight="10390" xr2:uid="{E094D080-3319-4F65-806B-502944EB452C}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11170" xr2:uid="{E094D080-3319-4F65-806B-502944EB452C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1977,25 +1977,25 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M62"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="21" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="52.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.85546875" style="3"/>
+    <col min="1" max="1" width="18.36328125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.36328125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6328125" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.36328125" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.90625" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="52.90625" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.90625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="22.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" ht="22.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="4" t="s">
         <v>115</v>
       </c>
@@ -2011,7 +2011,7 @@
       <c r="H1" s="55"/>
       <c r="I1" s="56"/>
     </row>
-    <row r="2" spans="1:13" ht="19.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" ht="19.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="4" t="s">
         <v>114</v>
       </c>
@@ -2027,8 +2027,8 @@
       <c r="H2" s="75"/>
       <c r="I2" s="76"/>
     </row>
-    <row r="3" spans="1:13" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="1:13" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:13" ht="22" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="4" spans="1:13" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="72" t="s">
         <v>7</v>
       </c>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="H4" s="73"/>
     </row>
-    <row r="5" spans="1:13" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:13" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="7" t="s">
         <v>1</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:13" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
@@ -2083,7 +2083,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:13" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
@@ -2098,7 +2098,7 @@
       <c r="G7" s="8"/>
       <c r="H7" s="21"/>
     </row>
-    <row r="8" spans="1:13" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:13" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B8" s="10"/>
       <c r="C8" s="11"/>
       <c r="E8" s="12"/>
@@ -2106,7 +2106,7 @@
       <c r="G8" s="8"/>
       <c r="H8" s="21"/>
     </row>
-    <row r="9" spans="1:13" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:13" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="10"/>
       <c r="C9" s="11"/>
       <c r="E9" s="10"/>
@@ -2114,7 +2114,7 @@
       <c r="G9" s="8"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="1:13" ht="9.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:13" ht="9.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
       <c r="H10" s="10"/>
@@ -2122,7 +2122,7 @@
       <c r="J10" s="10"/>
       <c r="K10" s="13"/>
     </row>
-    <row r="11" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="54" t="s">
         <v>1</v>
       </c>
@@ -2139,7 +2139,7 @@
       <c r="L11" s="55"/>
       <c r="M11" s="56"/>
     </row>
-    <row r="12" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A12" s="14" t="s">
         <v>140</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="40.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" ht="40" customHeight="1" thickTop="1" x14ac:dyDescent="0.5">
       <c r="A13" s="22" t="s">
         <v>178</v>
       </c>
@@ -2219,7 +2219,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A14" s="28"/>
       <c r="B14" s="29"/>
       <c r="C14" s="30"/>
@@ -2246,7 +2246,7 @@
       <c r="L14" s="32"/>
       <c r="M14" s="33"/>
     </row>
-    <row r="15" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="28"/>
       <c r="B15" s="29"/>
       <c r="C15" s="30"/>
@@ -2273,7 +2273,7 @@
       <c r="L15" s="32"/>
       <c r="M15" s="33"/>
     </row>
-    <row r="16" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A16" s="28"/>
       <c r="B16" s="29"/>
       <c r="C16" s="30"/>
@@ -2288,7 +2288,7 @@
       <c r="L16" s="32"/>
       <c r="M16" s="33"/>
     </row>
-    <row r="17" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A17" s="28"/>
       <c r="B17" s="29"/>
       <c r="C17" s="30"/>
@@ -2303,7 +2303,7 @@
       <c r="L17" s="32"/>
       <c r="M17" s="33"/>
     </row>
-    <row r="18" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A18" s="28"/>
       <c r="B18" s="29"/>
       <c r="C18" s="30"/>
@@ -2320,7 +2320,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A19" s="28" t="s">
         <v>178</v>
       </c>
@@ -2359,7 +2359,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A20" s="28"/>
       <c r="B20" s="29"/>
       <c r="C20" s="30"/>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="M20" s="33"/>
     </row>
-    <row r="21" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A21" s="28"/>
       <c r="B21" s="29"/>
       <c r="C21" s="30"/>
@@ -2403,7 +2403,7 @@
       <c r="L21" s="32"/>
       <c r="M21" s="33"/>
     </row>
-    <row r="22" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A22" s="28"/>
       <c r="B22" s="29"/>
       <c r="C22" s="30"/>
@@ -2418,7 +2418,7 @@
       <c r="L22" s="46"/>
       <c r="M22" s="33"/>
     </row>
-    <row r="23" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A23" s="28"/>
       <c r="B23" s="29"/>
       <c r="C23" s="30"/>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="M23" s="33"/>
     </row>
-    <row r="24" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A24" s="28"/>
       <c r="B24" s="29"/>
       <c r="C24" s="30"/>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="M24" s="33"/>
     </row>
-    <row r="25" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A25" s="28"/>
       <c r="B25" s="29"/>
       <c r="C25" s="30"/>
@@ -2467,7 +2467,7 @@
       <c r="L25" s="32"/>
       <c r="M25" s="33"/>
     </row>
-    <row r="26" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A26" s="28"/>
       <c r="B26" s="29"/>
       <c r="C26" s="30"/>
@@ -2482,7 +2482,7 @@
       <c r="L26" s="32"/>
       <c r="M26" s="33"/>
     </row>
-    <row r="27" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A27" s="28"/>
       <c r="B27" s="29"/>
       <c r="C27" s="30"/>
@@ -2497,7 +2497,7 @@
       <c r="L27" s="32"/>
       <c r="M27" s="33"/>
     </row>
-    <row r="28" spans="1:13" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="35"/>
       <c r="B28" s="36"/>
       <c r="C28" s="37"/>
@@ -2512,7 +2512,7 @@
       <c r="L28" s="39"/>
       <c r="M28" s="40"/>
     </row>
-    <row r="29" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="54" t="s">
         <v>156</v>
       </c>
@@ -2529,7 +2529,7 @@
       <c r="L29" s="55"/>
       <c r="M29" s="56"/>
     </row>
-    <row r="30" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A30" s="16" t="s">
         <v>157</v>
       </c>
@@ -2548,7 +2548,7 @@
       <c r="L30" s="77"/>
       <c r="M30" s="77"/>
     </row>
-    <row r="31" spans="1:13" ht="40.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" ht="40" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A31" s="17" t="str" cm="1">
         <f t="array" ref="A31">IFERROR(_xlfn.UNIQUE(_xlfn._xlws.FILTER(G13:G28,G13:G28&lt;&gt;"")),"")</f>
         <v>UNSEL</v>
@@ -2569,7 +2569,7 @@
       <c r="L31" s="78"/>
       <c r="M31" s="79"/>
     </row>
-    <row r="32" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="18"/>
       <c r="B32" s="63" t="str">
         <f>IF(A32&lt;&gt;"",_xlfn.XLOOKUP(A32,Colors[Colors],Colors[Description],"",0),"")</f>
@@ -2587,7 +2587,7 @@
       <c r="L32" s="63"/>
       <c r="M32" s="64"/>
     </row>
-    <row r="33" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="18"/>
       <c r="B33" s="63" t="str">
         <f>IF(A33&lt;&gt;"",_xlfn.XLOOKUP(A33,Colors[Colors],Colors[Description],"",0),"")</f>
@@ -2605,7 +2605,7 @@
       <c r="L33" s="63"/>
       <c r="M33" s="64"/>
     </row>
-    <row r="34" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="18"/>
       <c r="B34" s="63" t="str">
         <f>IF(A34&lt;&gt;"",_xlfn.XLOOKUP(A34,Colors[Colors],Colors[Description],"",0),"")</f>
@@ -2623,7 +2623,7 @@
       <c r="L34" s="63"/>
       <c r="M34" s="64"/>
     </row>
-    <row r="35" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="18"/>
       <c r="B35" s="63" t="str">
         <f>IF(A35&lt;&gt;"",_xlfn.XLOOKUP(A35,Colors[Colors],Colors[Description],"",0),"")</f>
@@ -2641,7 +2641,7 @@
       <c r="L35" s="63"/>
       <c r="M35" s="64"/>
     </row>
-    <row r="36" spans="1:13" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A36" s="19"/>
       <c r="B36" s="65" t="str">
         <f>IF(A36&lt;&gt;"",_xlfn.XLOOKUP(A36,Colors[Colors],Colors[Description],"",0),"")</f>
@@ -2659,7 +2659,7 @@
       <c r="L36" s="65"/>
       <c r="M36" s="66"/>
     </row>
-    <row r="37" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="54" t="s">
         <v>141</v>
       </c>
@@ -2676,7 +2676,7 @@
       <c r="L37" s="55"/>
       <c r="M37" s="56"/>
     </row>
-    <row r="38" spans="1:13" ht="40.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" ht="40" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A38" s="67" t="s">
         <v>177</v>
       </c>
@@ -2693,7 +2693,7 @@
       <c r="L38" s="61"/>
       <c r="M38" s="62"/>
     </row>
-    <row r="39" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="68"/>
       <c r="B39" s="52"/>
       <c r="C39" s="52"/>
@@ -2708,7 +2708,7 @@
       <c r="L39" s="52"/>
       <c r="M39" s="53"/>
     </row>
-    <row r="40" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="68"/>
       <c r="B40" s="52"/>
       <c r="C40" s="52"/>
@@ -2723,7 +2723,7 @@
       <c r="L40" s="52"/>
       <c r="M40" s="53"/>
     </row>
-    <row r="41" spans="1:13" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A41" s="68"/>
       <c r="B41" s="52"/>
       <c r="C41" s="52"/>
@@ -2738,7 +2738,7 @@
       <c r="L41" s="52"/>
       <c r="M41" s="53"/>
     </row>
-    <row r="42" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="54" t="s">
         <v>8</v>
       </c>
@@ -2755,7 +2755,7 @@
       <c r="L42" s="55"/>
       <c r="M42" s="56"/>
     </row>
-    <row r="43" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A43" s="14"/>
       <c r="B43" s="14" t="s">
         <v>107</v>
@@ -2780,7 +2780,7 @@
       <c r="L43" s="58"/>
       <c r="M43" s="59"/>
     </row>
-    <row r="44" spans="1:13" ht="40.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" ht="40" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A44" s="41"/>
       <c r="B44" s="42"/>
       <c r="C44" s="42">
@@ -2801,7 +2801,7 @@
       <c r="L44" s="61"/>
       <c r="M44" s="62"/>
     </row>
-    <row r="45" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="44"/>
       <c r="B45" s="30"/>
       <c r="C45" s="30"/>
@@ -2816,7 +2816,7 @@
       <c r="L45" s="52"/>
       <c r="M45" s="53"/>
     </row>
-    <row r="46" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="44"/>
       <c r="B46" s="30"/>
       <c r="C46" s="30"/>
@@ -2831,7 +2831,7 @@
       <c r="L46" s="52"/>
       <c r="M46" s="53"/>
     </row>
-    <row r="47" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="44"/>
       <c r="B47" s="30"/>
       <c r="C47" s="30"/>
@@ -2846,7 +2846,7 @@
       <c r="L47" s="52"/>
       <c r="M47" s="53"/>
     </row>
-    <row r="48" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="44"/>
       <c r="B48" s="30"/>
       <c r="C48" s="30"/>
@@ -2861,7 +2861,7 @@
       <c r="L48" s="52"/>
       <c r="M48" s="53"/>
     </row>
-    <row r="49" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="44"/>
       <c r="B49" s="30"/>
       <c r="C49" s="30"/>
@@ -2876,7 +2876,7 @@
       <c r="L49" s="52"/>
       <c r="M49" s="53"/>
     </row>
-    <row r="50" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="44"/>
       <c r="B50" s="30"/>
       <c r="C50" s="30"/>
@@ -2891,7 +2891,7 @@
       <c r="L50" s="52"/>
       <c r="M50" s="53"/>
     </row>
-    <row r="51" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="44"/>
       <c r="B51" s="30"/>
       <c r="C51" s="30"/>
@@ -2906,7 +2906,7 @@
       <c r="L51" s="52"/>
       <c r="M51" s="53"/>
     </row>
-    <row r="52" spans="1:13" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A52" s="45"/>
       <c r="B52" s="37"/>
       <c r="C52" s="37"/>
@@ -2921,7 +2921,7 @@
       <c r="L52" s="49"/>
       <c r="M52" s="50"/>
     </row>
-    <row r="53" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="54" t="s">
         <v>9</v>
       </c>
@@ -2938,7 +2938,7 @@
       <c r="L53" s="55"/>
       <c r="M53" s="56"/>
     </row>
-    <row r="54" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A54" s="14"/>
       <c r="B54" s="14" t="s">
         <v>107</v>
@@ -2963,7 +2963,7 @@
       <c r="L54" s="58"/>
       <c r="M54" s="59"/>
     </row>
-    <row r="55" spans="1:13" ht="40.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" ht="40" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A55" s="41"/>
       <c r="B55" s="42"/>
       <c r="C55" s="42"/>
@@ -2978,7 +2978,7 @@
       <c r="L55" s="61"/>
       <c r="M55" s="62"/>
     </row>
-    <row r="56" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="44"/>
       <c r="B56" s="30"/>
       <c r="C56" s="30"/>
@@ -2993,7 +2993,7 @@
       <c r="L56" s="52"/>
       <c r="M56" s="53"/>
     </row>
-    <row r="57" spans="1:13" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A57" s="44"/>
       <c r="B57" s="30"/>
       <c r="C57" s="30"/>
@@ -3008,7 +3008,7 @@
       <c r="L57" s="49"/>
       <c r="M57" s="50"/>
     </row>
-    <row r="58" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="54" t="s">
         <v>19</v>
       </c>
@@ -3025,7 +3025,7 @@
       <c r="L58" s="55"/>
       <c r="M58" s="56"/>
     </row>
-    <row r="59" spans="1:13" ht="40.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:13" ht="40" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A59" s="14"/>
       <c r="B59" s="14" t="s">
         <v>107</v>
@@ -3050,7 +3050,7 @@
       <c r="L59" s="58"/>
       <c r="M59" s="59"/>
     </row>
-    <row r="60" spans="1:13" ht="40.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" ht="40" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A60" s="41"/>
       <c r="B60" s="42" t="s">
         <v>135</v>
@@ -3073,7 +3073,7 @@
       <c r="L60" s="61"/>
       <c r="M60" s="62"/>
     </row>
-    <row r="61" spans="1:13" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A61" s="45"/>
       <c r="B61" s="37"/>
       <c r="C61" s="37"/>
@@ -3088,7 +3088,7 @@
       <c r="L61" s="49"/>
       <c r="M61" s="50"/>
     </row>
-    <row r="62" spans="1:13" ht="21.75" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="62" spans="1:13" ht="21.5" thickTop="1" x14ac:dyDescent="0.5"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="1CC3n0ipDpk6c381gKxkr7OO6P5vEU3nlZFR+vtG+1FlJqeGd8RPXsVJ6NyWD3qwHko2nHIsSrzn41DhANG/4w==" saltValue="9S3PHMnQi/Bv80wTCQbelg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="41">
@@ -3181,23 +3181,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D8A0A11-4DA6-418B-866F-D5B6956565A1}">
   <dimension ref="A1:W20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.54296875" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="234.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.28515625" customWidth="1"/>
-    <col min="17" max="17" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="234.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.36328125" customWidth="1"/>
+    <col min="17" max="17" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.6328125" customWidth="1"/>
     <col min="21" max="21" width="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.7109375" customWidth="1"/>
+    <col min="23" max="23" width="8.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -3285,7 +3285,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -3329,7 +3329,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -3373,7 +3373,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -3417,7 +3417,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -3458,7 +3458,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -3496,7 +3496,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -3534,7 +3534,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -3572,7 +3572,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -3607,7 +3607,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>30</v>
       </c>
@@ -3627,7 +3627,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>31</v>
       </c>
@@ -3647,7 +3647,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="M13" t="s">
         <v>72</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="M14" t="s">
         <v>167</v>
       </c>
@@ -3666,7 +3666,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>170</v>
       </c>
@@ -3677,27 +3677,27 @@
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="M16" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="17" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M17" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M18" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M19" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M20" t="s">
         <v>76</v>
       </c>

</xml_diff>